<commit_message>
Remplace le pseudonyme par le nom de l'auteur (Jaurès DAA-HINGBANON)
</commit_message>
<xml_diff>
--- a/livrables/05_Tableaux/Indicateurs_diagnostic_ZAN_Rouen.xlsx
+++ b/livrables/05_Tableaux/Indicateurs_diagnostic_ZAN_Rouen.xlsx
@@ -22,7 +22,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Zones AU'!$A$3:$O$130</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Gisements'!$A$3:$P$369</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Transitions OCS GE'!$A$3:$H$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Dictionnaire'!$A$3:$D$178</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Dictionnaire'!$A$3:$D$190</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -486,7 +486,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Sources : Cerema 2011-2025, IGN OCS GE 2019-2022, Géoportail de l'Urbanisme, RPG 2024. Réalisation : Jauresmas, 09/10/2026</t>
+          <t>Sources : Cerema 2011-2025, IGN OCS GE 2019-2022, Géoportail de l'Urbanisme, RPG 2024. Réalisation : Jaurès DAA-HINGBANON, 13/10/2026</t>
         </is>
       </c>
     </row>
@@ -817,7 +817,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Sources : Cerema 2011-2025, IGN OCS GE 2019-2022, Géoportail de l'Urbanisme, RPG 2024. Réalisation : Jauresmas, 09/10/2026</t>
+          <t>Sources : Cerema 2011-2025, IGN OCS GE 2019-2022, Géoportail de l'Urbanisme, RPG 2024. Réalisation : Jaurès DAA-HINGBANON, 13/10/2026</t>
         </is>
       </c>
     </row>
@@ -14189,7 +14189,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Sources : Cerema 2011-2025, IGN OCS GE 2019-2022, Géoportail de l'Urbanisme, RPG 2024. Réalisation : Jauresmas, 09/10/2026</t>
+          <t>Sources : Cerema 2011-2025, IGN OCS GE 2019-2022, Géoportail de l'Urbanisme, RPG 2024. Réalisation : Jaurès DAA-HINGBANON, 13/10/2026</t>
         </is>
       </c>
     </row>
@@ -14594,7 +14594,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Sources : Cerema 2011-2025, IGN OCS GE 2019-2022, Géoportail de l'Urbanisme, RPG 2024. Réalisation : Jauresmas, 09/10/2026</t>
+          <t>Sources : Cerema 2011-2025, IGN OCS GE 2019-2022, Géoportail de l'Urbanisme, RPG 2024. Réalisation : Jaurès DAA-HINGBANON, 13/10/2026</t>
         </is>
       </c>
     </row>
@@ -22973,7 +22973,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Sources : Cerema 2011-2025, IGN OCS GE 2019-2022, Géoportail de l'Urbanisme, RPG 2024. Réalisation : Jauresmas, 09/10/2026</t>
+          <t>Sources : Cerema 2011-2025, IGN OCS GE 2019-2022, Géoportail de l'Urbanisme, RPG 2024. Réalisation : Jaurès DAA-HINGBANON, 13/10/2026</t>
         </is>
       </c>
     </row>
@@ -44526,7 +44526,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Sources : Cerema 2011-2025, IGN OCS GE 2019-2022, Géoportail de l'Urbanisme, RPG 2024. Réalisation : Jauresmas, 09/10/2026</t>
+          <t>Sources : Cerema 2011-2025, IGN OCS GE 2019-2022, Géoportail de l'Urbanisme, RPG 2024. Réalisation : Jaurès DAA-HINGBANON, 13/10/2026</t>
         </is>
       </c>
     </row>
@@ -44780,7 +44780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D178"/>
+  <dimension ref="A1:D190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -44799,7 +44799,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Sources : Cerema 2011-2025, IGN OCS GE 2019-2022, Géoportail de l'Urbanisme, RPG 2024. Réalisation : Jauresmas, 09/10/2026</t>
+          <t>Sources : Cerema 2011-2025, IGN OCS GE 2019-2022, Géoportail de l'Urbanisme, RPG 2024. Réalisation : Jaurès DAA-HINGBANON, 13/10/2026</t>
         </is>
       </c>
     </row>
@@ -48675,8 +48675,272 @@
         </is>
       </c>
     </row>
+    <row r="179">
+      <c r="A179" s="4" t="inlineStr">
+        <is>
+          <t>cadastre_parcelles_etude</t>
+        </is>
+      </c>
+      <c r="B179" s="4" t="inlineStr">
+        <is>
+          <t>idu</t>
+        </is>
+      </c>
+      <c r="C179" s="4" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="D179" s="4" t="inlineStr">
+        <is>
+          <t>Identifiant cadastral de la parcelle</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="4" t="inlineStr">
+        <is>
+          <t>cadastre_parcelles_etude</t>
+        </is>
+      </c>
+      <c r="B180" s="4" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+      <c r="C180" s="4" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="D180" s="4" t="inlineStr">
+        <is>
+          <t>Section cadastrale</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="4" t="inlineStr">
+        <is>
+          <t>cadastre_parcelles_etude</t>
+        </is>
+      </c>
+      <c r="B181" s="4" t="inlineStr">
+        <is>
+          <t>numero</t>
+        </is>
+      </c>
+      <c r="C181" s="4" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="D181" s="4" t="inlineStr">
+        <is>
+          <t>Numéro de parcelle</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="4" t="inlineStr">
+        <is>
+          <t>cadastre_parcelles_etude</t>
+        </is>
+      </c>
+      <c r="B182" s="4" t="inlineStr">
+        <is>
+          <t>contenance</t>
+        </is>
+      </c>
+      <c r="C182" s="4" t="inlineStr">
+        <is>
+          <t>float64</t>
+        </is>
+      </c>
+      <c r="D182" s="4" t="inlineStr">
+        <is>
+          <t>Contenance cadastrale (m²)</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="4" t="inlineStr">
+        <is>
+          <t>cadastre_parcelles_etude</t>
+        </is>
+      </c>
+      <c r="B183" s="4" t="inlineStr">
+        <is>
+          <t>code_insee</t>
+        </is>
+      </c>
+      <c r="C183" s="4" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="D183" s="4" t="inlineStr">
+        <is>
+          <t>Code INSEE de la commune</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="4" t="inlineStr">
+        <is>
+          <t>bdtopo_batiments_etude</t>
+        </is>
+      </c>
+      <c r="B184" s="4" t="inlineStr">
+        <is>
+          <t>cleabs</t>
+        </is>
+      </c>
+      <c r="C184" s="4" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="D184" s="4" t="inlineStr">
+        <is>
+          <t>Identifiant BD TOPO</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="4" t="inlineStr">
+        <is>
+          <t>bdtopo_batiments_etude</t>
+        </is>
+      </c>
+      <c r="B185" s="4" t="inlineStr">
+        <is>
+          <t>nature</t>
+        </is>
+      </c>
+      <c r="C185" s="4" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="D185" s="4" t="inlineStr">
+        <is>
+          <t>Nature du bâtiment</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="4" t="inlineStr">
+        <is>
+          <t>bdtopo_batiments_etude</t>
+        </is>
+      </c>
+      <c r="B186" s="4" t="inlineStr">
+        <is>
+          <t>usage_1</t>
+        </is>
+      </c>
+      <c r="C186" s="4" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="D186" s="4" t="inlineStr">
+        <is>
+          <t>Usage principal du bâtiment</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="4" t="inlineStr">
+        <is>
+          <t>bdtopo_batiments_etude</t>
+        </is>
+      </c>
+      <c r="B187" s="4" t="inlineStr">
+        <is>
+          <t>construction_legere</t>
+        </is>
+      </c>
+      <c r="C187" s="4" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="D187" s="4" t="inlineStr">
+        <is>
+          <t>Construction légère (1) ou non (0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="4" t="inlineStr">
+        <is>
+          <t>bdtopo_batiments_etude</t>
+        </is>
+      </c>
+      <c r="B188" s="4" t="inlineStr">
+        <is>
+          <t>nombre_de_logements</t>
+        </is>
+      </c>
+      <c r="C188" s="4" t="inlineStr">
+        <is>
+          <t>float64</t>
+        </is>
+      </c>
+      <c r="D188" s="4" t="inlineStr">
+        <is>
+          <t>Nombre de logements</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="4" t="inlineStr">
+        <is>
+          <t>bdtopo_batiments_etude</t>
+        </is>
+      </c>
+      <c r="B189" s="4" t="inlineStr">
+        <is>
+          <t>hauteur</t>
+        </is>
+      </c>
+      <c r="C189" s="4" t="inlineStr">
+        <is>
+          <t>float64</t>
+        </is>
+      </c>
+      <c r="D189" s="4" t="inlineStr">
+        <is>
+          <t>Hauteur du bâtiment (m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="4" t="inlineStr">
+        <is>
+          <t>bdtopo_batiments_etude</t>
+        </is>
+      </c>
+      <c r="B190" s="4" t="inlineStr">
+        <is>
+          <t>code_insee</t>
+        </is>
+      </c>
+      <c r="C190" s="4" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="D190" s="4" t="inlineStr">
+        <is>
+          <t>Code INSEE de la commune</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:D178"/>
+  <autoFilter ref="A3:D190"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>